<commit_message>
Update fsh-generated and output artifacts from SUSHI and IG Publisher
Regenerated fsh-generated/ resources and output/ HTML/JSON/TTL files
reflecting all ballot reconciliation changes in this branch.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/CodeSystem-EndpointPayloadTypeCS.xlsx
+++ b/output/CodeSystem-EndpointPayloadTypeCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.1.1</t>
+    <t>2.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-17T14:48:28-05:00</t>
+    <t>2026-03-17T22:49:33-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>